<commit_message>
Docs: README.md, 현황 excel 업데이트
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\비전공_18회차\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560AD5D8-B1F0-4281-A104-F028AF23D883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="636" yWindow="396" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,15 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -368,7 +360,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="16">
     <font>
       <sz val="11"/>
@@ -650,7 +642,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -675,6 +667,9 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -684,10 +679,13 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -714,17 +712,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -752,15 +741,15 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp11.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp12.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp13.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp14.xml><?xml version="1.0" encoding="utf-8"?>
@@ -768,7 +757,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp16.xml><?xml version="1.0" encoding="utf-8"?>
@@ -776,7 +765,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp17.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp18.xml><?xml version="1.0" encoding="utf-8"?>
@@ -784,7 +773,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp19.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -804,7 +793,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp23.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp24.xml><?xml version="1.0" encoding="utf-8"?>
@@ -902,7 +891,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -969,7 +958,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1036,7 +1025,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1103,7 +1092,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1170,7 +1159,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1237,7 +1226,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1304,7 +1293,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193430</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1371,7 +1360,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193430</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1438,7 +1427,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1505,7 +1494,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1572,7 +1561,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1639,7 +1628,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>193431</xdr:rowOff>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1700,13 +1689,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>5</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1767,13 +1756,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>5</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1834,13 +1823,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1901,13 +1890,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1968,13 +1957,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2035,13 +2024,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2102,13 +2091,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>9526</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2169,13 +2158,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>9526</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2236,13 +2225,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>10</xdr:row>
-          <xdr:rowOff>9524</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2303,13 +2292,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>10</xdr:row>
-          <xdr:rowOff>9524</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2370,13 +2359,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>10</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2437,13 +2426,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>10</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2504,13 +2493,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2571,13 +2560,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>11</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2638,13 +2627,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>9526</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2705,13 +2694,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>12</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>9526</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2772,13 +2761,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>9524</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2839,13 +2828,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>13</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>9524</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2906,13 +2895,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2973,13 +2962,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>14</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3040,13 +3029,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3107,13 +3096,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>15</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3174,13 +3163,13 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>17</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3241,13 +3230,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>38100</xdr:colOff>
           <xdr:row>16</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>266700</xdr:colOff>
           <xdr:row>17</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3302,10 +3291,6 @@
     <mc:Fallback/>
   </mc:AlternateContent>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3604,47 +3589,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <cols>
-    <col min="1" max="1" width="25.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="3.625" customWidth="1"/>
-    <col min="5" max="6" width="10.625" customWidth="1"/>
+    <col min="1" max="1" width="25.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="3.59765625" customWidth="1"/>
+    <col min="5" max="6" width="10.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19.5">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="20.399999999999999">
+      <c r="A1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="27" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="16" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="16"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
@@ -3666,14 +3651,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="22.5">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:6" ht="21.6">
+      <c r="A5" s="19" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="22"/>
+      <c r="C5" s="8"/>
       <c r="D5" s="5"/>
       <c r="E5" s="6" t="s">
         <v>24</v>
@@ -3683,11 +3668,11 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="17"/>
+      <c r="A6" s="19"/>
       <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="22"/>
+      <c r="C6" s="8"/>
       <c r="D6" s="5"/>
       <c r="E6" s="6" t="s">
         <v>26</v>
@@ -3697,11 +3682,11 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="17"/>
+      <c r="A7" s="19"/>
       <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="22"/>
+      <c r="C7" s="8"/>
       <c r="D7" s="5"/>
       <c r="E7" s="6" t="s">
         <v>27</v>
@@ -3711,11 +3696,11 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="17"/>
+      <c r="A8" s="19"/>
       <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="22"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="5"/>
       <c r="E8" s="6" t="s">
         <v>28</v>
@@ -3725,11 +3710,11 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="17"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="8"/>
       <c r="D9" s="5"/>
       <c r="E9" s="6" t="s">
         <v>29</v>
@@ -3739,11 +3724,11 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="17"/>
+      <c r="A10" s="19"/>
       <c r="B10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="22"/>
+      <c r="C10" s="8"/>
       <c r="D10" s="5"/>
       <c r="E10" s="6" t="s">
         <v>30</v>
@@ -3753,11 +3738,11 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="17"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="22"/>
+      <c r="C11" s="8"/>
       <c r="D11" s="5"/>
       <c r="E11" s="6" t="s">
         <v>31</v>
@@ -3767,11 +3752,11 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="17"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="22"/>
+      <c r="C12" s="8"/>
       <c r="D12" s="5"/>
       <c r="E12" s="6" t="s">
         <v>32</v>
@@ -3781,11 +3766,11 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="17"/>
+      <c r="A13" s="19"/>
       <c r="B13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="22"/>
+      <c r="C13" s="8"/>
       <c r="D13" s="5"/>
       <c r="E13" s="6" t="s">
         <v>33</v>
@@ -3795,11 +3780,11 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="17"/>
+      <c r="A14" s="19"/>
       <c r="B14" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="22"/>
+      <c r="C14" s="8"/>
       <c r="D14" s="5"/>
       <c r="E14" s="6" t="s">
         <v>34</v>
@@ -3809,11 +3794,11 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="17"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="8"/>
       <c r="D15" s="5"/>
       <c r="E15" s="6" t="s">
         <v>35</v>
@@ -3823,11 +3808,11 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="17"/>
+      <c r="A16" s="19"/>
       <c r="B16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="22"/>
+      <c r="C16" s="8"/>
       <c r="D16" s="5"/>
       <c r="E16" s="6" t="s">
         <v>36</v>
@@ -3837,11 +3822,11 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="17"/>
+      <c r="A17" s="19"/>
       <c r="B17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="22"/>
+      <c r="C17" s="8"/>
       <c r="D17" s="5"/>
       <c r="E17" s="6" t="s">
         <v>37</v>
@@ -3851,52 +3836,52 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="23"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -4192,13 +4177,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>5</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>6</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4214,13 +4199,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>5</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>6</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4236,13 +4221,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>6</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>7</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4258,13 +4243,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>6</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>7</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4280,13 +4265,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>7</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4302,13 +4287,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>7</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4324,13 +4309,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>9</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4346,13 +4331,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>9</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4368,13 +4353,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>9</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>10</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4390,13 +4375,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>9</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>10</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4412,13 +4397,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>10</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>11</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4434,13 +4419,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>10</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>11</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4456,13 +4441,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>11</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>12</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4478,13 +4463,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>11</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>12</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4500,13 +4485,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>12</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>13</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4522,13 +4507,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>12</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>13</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4544,13 +4529,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>13</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>14</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4566,13 +4551,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>13</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>14</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4588,13 +4573,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>14</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>15</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4610,13 +4595,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>14</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>15</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4632,13 +4617,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>15</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>16</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4654,13 +4639,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>15</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>16</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4676,13 +4661,13 @@
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>16</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>17</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4698,13 +4683,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>16</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>266700</xdr:colOff>
                     <xdr:row>17</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>

<commit_message>
Docs: 02_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D16B06-029F-4591-B53B-511C03E4CBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862EE777-7F79-4715-976D-F154541DFF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -753,7 +753,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp14.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 03_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862EE777-7F79-4715-976D-F154541DFF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F5524-801A-4526-8D72-BCCF9282A077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -761,7 +761,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp16.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp17.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 04_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F5524-801A-4526-8D72-BCCF9282A077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA188ED-E863-4048-8D31-2729C84BC2E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp18.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp19.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 05_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA188ED-E863-4048-8D31-2729C84BC2E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3F0D91-5352-45A7-A268-2D098C67CDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -781,7 +781,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp20.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp21.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 07_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3F0D91-5352-45A7-A268-2D098C67CDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C013E6-2F8D-4C08-B395-263BDCF38C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -797,7 +797,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp24.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp25.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 09_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C013E6-2F8D-4C08-B395-263BDCF38C03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CB2ABE-9A84-46ED-BA2D-AEA29C941A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -809,7 +809,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp27.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp28.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 09_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CB2ABE-9A84-46ED-BA2D-AEA29C941A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684638EA-5C88-400C-96A6-FFC126E770CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -813,7 +813,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp28.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp29.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 06_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684638EA-5C88-400C-96A6-FFC126E770CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D0D216-AACD-4DD1-AFD4-B02902BED3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -785,7 +785,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp21.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp22.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 06_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D0D216-AACD-4DD1-AFD4-B02902BED3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC4A1A2-4675-4042-9A3B-BC1E3C22C2C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -789,7 +789,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp22.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp23.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 10_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC4A1A2-4675-4042-9A3B-BC1E3C22C2C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565F0C26-D283-4EFB-A46B-CC487B9E3E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -817,7 +817,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp29.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 10_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565F0C26-D283-4EFB-A46B-CC487B9E3E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6735473-F34F-4E70-94D9-5DA9B97F6CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10836" yWindow="456" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6084" yWindow="1440" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -825,7 +825,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp30.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp31.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 11_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6735473-F34F-4E70-94D9-5DA9B97F6CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B476094-0459-492F-A6AF-EA4445E2E4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6084" yWindow="1440" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -829,7 +829,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp31.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp32.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 11_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B476094-0459-492F-A6AF-EA4445E2E4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580AF352-8BAF-4978-9F02-17890B6FBAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6084" yWindow="1440" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -833,7 +833,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp32.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp33.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 12_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580AF352-8BAF-4978-9F02-17890B6FBAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C4909C-5138-4006-81D9-4F7866B90A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6084" yWindow="1440" windowWidth="10488" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="672" yWindow="744" windowWidth="7716" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -837,7 +837,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp33.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp34.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 12_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C4909C-5138-4006-81D9-4F7866B90A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14D9143-4ED0-4532-AAAC-4DAEC59E07A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="672" yWindow="744" windowWidth="7716" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -841,7 +841,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp34.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp35.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 13_java(기본) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14D9143-4ED0-4532-AAAC-4DAEC59E07A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A1CBD2-A6D6-4093-9EAA-57D915678FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="672" yWindow="744" windowWidth="7716" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -845,7 +845,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp35.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp36.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docs: 13_java(심화) 과제 완료
</commit_message>
<xml_diff>
--- a/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term2/18회차_실습체크리스트_김윤지.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A1CBD2-A6D6-4093-9EAA-57D915678FA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD50870B-E1AD-47BD-92D4-3019E9E8245B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="672" yWindow="744" windowWidth="7716" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -849,7 +849,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp36.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>